<commit_message>
Analiza modelului final (explainability). Interpretarea rezultatelor. Începerea structurării documentației
</commit_message>
<xml_diff>
--- a/rezultate_brute_modele.xlsx
+++ b/rezultate_brute_modele.xlsx
@@ -467,30 +467,30 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Random Forest</t>
+          <t>ElasticNet</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>0.8944</v>
+        <v>0.9963</v>
       </c>
       <c r="D2" t="n">
-        <v>1.5697</v>
+        <v>0.0065</v>
       </c>
       <c r="E2" t="n">
-        <v>1.2174</v>
+        <v>0.0052</v>
       </c>
       <c r="F2" t="n">
-        <v>2.4639</v>
+        <v>0</v>
       </c>
       <c r="G2" t="n">
-        <v>0.7512</v>
+        <v>0.9913</v>
       </c>
       <c r="H2" t="n">
-        <v>0.0488</v>
+        <v>0.0038</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>{'max_depth': None, 'min_samples_split': 2, 'n_estimators': 100}</t>
+          <t>{'alpha': 0.001, 'l1_ratio': 0.2}</t>
         </is>
       </c>
     </row>
@@ -500,30 +500,30 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>AdaBoost</t>
+          <t>Ridge Regression</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>0.8918</v>
+        <v>0.9962</v>
       </c>
       <c r="D3" t="n">
-        <v>1.5885</v>
+        <v>0.0065</v>
       </c>
       <c r="E3" t="n">
-        <v>1.2696</v>
+        <v>0.0052</v>
       </c>
       <c r="F3" t="n">
-        <v>2.5234</v>
+        <v>0</v>
       </c>
       <c r="G3" t="n">
-        <v>0.739</v>
+        <v>0.9913999999999999</v>
       </c>
       <c r="H3" t="n">
-        <v>0.0372</v>
+        <v>0.0039</v>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>{'learning_rate': 1.0, 'n_estimators': 200}</t>
+          <t>{'alpha': 1}</t>
         </is>
       </c>
     </row>
@@ -533,30 +533,30 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Ridge Regression</t>
+          <t>Lasso Regression</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>0.8733</v>
+        <v>0.9954</v>
       </c>
       <c r="D4" t="n">
-        <v>1.7189</v>
+        <v>0.0072</v>
       </c>
       <c r="E4" t="n">
-        <v>1.2705</v>
+        <v>0.0058</v>
       </c>
       <c r="F4" t="n">
-        <v>2.9546</v>
+        <v>0.0001</v>
       </c>
       <c r="G4" t="n">
-        <v>0.7692</v>
+        <v>0.9909</v>
       </c>
       <c r="H4" t="n">
-        <v>0.043</v>
+        <v>0.004</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>{'alpha': 10}</t>
+          <t>{'alpha': 0.001}</t>
         </is>
       </c>
     </row>
@@ -566,30 +566,30 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Gradient Boosting</t>
+          <t>SVR</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>0.8715000000000001</v>
+        <v>0.9953</v>
       </c>
       <c r="D5" t="n">
-        <v>1.7315</v>
+        <v>0.0073</v>
       </c>
       <c r="E5" t="n">
-        <v>1.3257</v>
+        <v>0.0056</v>
       </c>
       <c r="F5" t="n">
-        <v>2.9982</v>
+        <v>0.0001</v>
       </c>
       <c r="G5" t="n">
-        <v>0.7654</v>
+        <v>0.9903999999999999</v>
       </c>
       <c r="H5" t="n">
-        <v>0.0546</v>
+        <v>0.0038</v>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>{'learning_rate': 0.1, 'max_depth': 3, 'n_estimators': 50}</t>
+          <t>{'C': 0.1, 'epsilon': 0.01, 'kernel': 'linear'}</t>
         </is>
       </c>
     </row>
@@ -599,30 +599,30 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>ElasticNet</t>
+          <t>Gradient Boosting</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>0.8711</v>
+        <v>0.9568</v>
       </c>
       <c r="D6" t="n">
-        <v>1.734</v>
+        <v>0.0221</v>
       </c>
       <c r="E6" t="n">
-        <v>1.2775</v>
+        <v>0.0168</v>
       </c>
       <c r="F6" t="n">
-        <v>3.0068</v>
+        <v>0.0005</v>
       </c>
       <c r="G6" t="n">
-        <v>0.77</v>
+        <v>0.9503</v>
       </c>
       <c r="H6" t="n">
-        <v>0.0453</v>
+        <v>0.0105</v>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>{'alpha': 0.1, 'l1_ratio': 0.2}</t>
+          <t>{'learning_rate': 0.05, 'max_depth': 3, 'n_estimators': 200}</t>
         </is>
       </c>
     </row>
@@ -632,30 +632,30 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Lasso Regression</t>
+          <t>Extra Trees</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>0.8709</v>
+        <v>0.9453</v>
       </c>
       <c r="D7" t="n">
-        <v>1.7351</v>
+        <v>0.0249</v>
       </c>
       <c r="E7" t="n">
-        <v>1.2851</v>
+        <v>0.0194</v>
       </c>
       <c r="F7" t="n">
-        <v>3.0105</v>
+        <v>0.0005999999999999999</v>
       </c>
       <c r="G7" t="n">
-        <v>0.7685</v>
+        <v>0.9634</v>
       </c>
       <c r="H7" t="n">
-        <v>0.0455</v>
+        <v>0.0198</v>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>{'alpha': 0.1}</t>
+          <t>{'max_depth': 10, 'min_samples_split': 2, 'n_estimators': 100}</t>
         </is>
       </c>
     </row>
@@ -665,30 +665,30 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>SVR</t>
+          <t>Random Forest</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>0.8671</v>
+        <v>0.9316</v>
       </c>
       <c r="D8" t="n">
-        <v>1.7605</v>
+        <v>0.0278</v>
       </c>
       <c r="E8" t="n">
-        <v>1.2942</v>
+        <v>0.0201</v>
       </c>
       <c r="F8" t="n">
-        <v>3.0994</v>
+        <v>0.0008</v>
       </c>
       <c r="G8" t="n">
-        <v>0.7647</v>
+        <v>0.9261</v>
       </c>
       <c r="H8" t="n">
-        <v>0.0358</v>
+        <v>0.0201</v>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>{'C': 1, 'epsilon': 0.5, 'kernel': 'linear'}</t>
+          <t>{'max_depth': 10, 'min_samples_split': 2, 'n_estimators': 200}</t>
         </is>
       </c>
     </row>
@@ -698,30 +698,30 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Extra Trees</t>
+          <t>AdaBoost</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>0.8471</v>
+        <v>0.9182</v>
       </c>
       <c r="D9" t="n">
-        <v>1.8883</v>
+        <v>0.0305</v>
       </c>
       <c r="E9" t="n">
-        <v>1.3312</v>
+        <v>0.0234</v>
       </c>
       <c r="F9" t="n">
-        <v>3.5657</v>
+        <v>0.0009</v>
       </c>
       <c r="G9" t="n">
-        <v>0.7762</v>
+        <v>0.9163</v>
       </c>
       <c r="H9" t="n">
-        <v>0.0323</v>
+        <v>0.0184</v>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>{'max_depth': None, 'min_samples_split': 2, 'n_estimators': 100}</t>
+          <t>{'learning_rate': 1.0, 'n_estimators': 200}</t>
         </is>
       </c>
     </row>
@@ -731,30 +731,30 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>KNN Regression</t>
+          <t>Decision Tree</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>0.806</v>
+        <v>0.8459</v>
       </c>
       <c r="D10" t="n">
-        <v>2.1271</v>
+        <v>0.0418</v>
       </c>
       <c r="E10" t="n">
-        <v>1.4703</v>
+        <v>0.0339</v>
       </c>
       <c r="F10" t="n">
-        <v>4.5246</v>
+        <v>0.0017</v>
       </c>
       <c r="G10" t="n">
-        <v>0.737</v>
+        <v>0.8544</v>
       </c>
       <c r="H10" t="n">
-        <v>0.0312</v>
+        <v>0.0397</v>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>{'metric': 'euclidean', 'n_neighbors': 10, 'weights': 'distance'}</t>
+          <t>{'max_depth': None, 'min_samples_leaf': 1, 'min_samples_split': 2}</t>
         </is>
       </c>
     </row>
@@ -764,30 +764,30 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Decision Tree</t>
+          <t>KNN Regression</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>0.7343</v>
+        <v>0.7766999999999999</v>
       </c>
       <c r="D11" t="n">
-        <v>2.4892</v>
+        <v>0.0503</v>
       </c>
       <c r="E11" t="n">
-        <v>1.5311</v>
+        <v>0.0372</v>
       </c>
       <c r="F11" t="n">
-        <v>6.196</v>
+        <v>0.0025</v>
       </c>
       <c r="G11" t="n">
-        <v>0.6264999999999999</v>
+        <v>0.8114</v>
       </c>
       <c r="H11" t="n">
-        <v>0.1306</v>
+        <v>0.0311</v>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>{'max_depth': 5, 'min_samples_leaf': 4, 'min_samples_split': 2}</t>
+          <t>{'metric': 'euclidean', 'n_neighbors': 5, 'weights': 'distance'}</t>
         </is>
       </c>
     </row>
@@ -853,30 +853,30 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Gradient Boosting</t>
+          <t>Ridge Regression</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>0.9877</v>
+        <v>1</v>
       </c>
       <c r="D2" t="n">
-        <v>0.2586</v>
+        <v>0</v>
       </c>
       <c r="E2" t="n">
-        <v>0.1326</v>
+        <v>0</v>
       </c>
       <c r="F2" t="n">
-        <v>0.0669</v>
+        <v>0</v>
       </c>
       <c r="G2" t="n">
-        <v>0.9841</v>
+        <v>1</v>
       </c>
       <c r="H2" t="n">
-        <v>0.0109</v>
+        <v>0</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>{'learning_rate': 0.1, 'max_depth': 3, 'n_estimators': 200}</t>
+          <t>{'alpha': 0.01}</t>
         </is>
       </c>
     </row>
@@ -886,30 +886,30 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Ridge Regression</t>
+          <t>ElasticNet</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>0.9867</v>
+        <v>0.9999</v>
       </c>
       <c r="D3" t="n">
-        <v>0.269</v>
+        <v>0.0005999999999999999</v>
       </c>
       <c r="E3" t="n">
-        <v>0.1881</v>
+        <v>0.0005</v>
       </c>
       <c r="F3" t="n">
-        <v>0.07240000000000001</v>
+        <v>0</v>
       </c>
       <c r="G3" t="n">
-        <v>0.9717</v>
+        <v>0.9999</v>
       </c>
       <c r="H3" t="n">
-        <v>0.0062</v>
+        <v>0</v>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>{'alpha': 1}</t>
+          <t>{'alpha': 0.001, 'l1_ratio': 0.2}</t>
         </is>
       </c>
     </row>
@@ -919,30 +919,30 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>ElasticNet</t>
+          <t>Lasso Regression</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>0.9866</v>
+        <v>0.9986</v>
       </c>
       <c r="D4" t="n">
-        <v>0.2692</v>
+        <v>0.0028</v>
       </c>
       <c r="E4" t="n">
-        <v>0.1882</v>
+        <v>0.0023</v>
       </c>
       <c r="F4" t="n">
-        <v>0.0725</v>
+        <v>0</v>
       </c>
       <c r="G4" t="n">
-        <v>0.9717</v>
+        <v>0.9986</v>
       </c>
       <c r="H4" t="n">
-        <v>0.0062</v>
+        <v>0.0002</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>{'alpha': 0.001, 'l1_ratio': 0.8}</t>
+          <t>{'alpha': 0.001}</t>
         </is>
       </c>
     </row>
@@ -952,30 +952,30 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Lasso Regression</t>
+          <t>SVR</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>0.9866</v>
+        <v>0.9963</v>
       </c>
       <c r="D5" t="n">
-        <v>0.2692</v>
+        <v>0.0045</v>
       </c>
       <c r="E5" t="n">
-        <v>0.1881</v>
+        <v>0.0036</v>
       </c>
       <c r="F5" t="n">
-        <v>0.0725</v>
+        <v>0</v>
       </c>
       <c r="G5" t="n">
-        <v>0.9717</v>
+        <v>0.9961</v>
       </c>
       <c r="H5" t="n">
-        <v>0.0062</v>
+        <v>0.0007</v>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>{'alpha': 0.001}</t>
+          <t>{'C': 0.1, 'epsilon': 0.01, 'kernel': 'linear'}</t>
         </is>
       </c>
     </row>
@@ -985,30 +985,30 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>SVR</t>
+          <t>Gradient Boosting</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>0.9865</v>
+        <v>0.9664</v>
       </c>
       <c r="D6" t="n">
-        <v>0.2711</v>
+        <v>0.0137</v>
       </c>
       <c r="E6" t="n">
-        <v>0.1839</v>
+        <v>0.009900000000000001</v>
       </c>
       <c r="F6" t="n">
-        <v>0.0735</v>
+        <v>0.0002</v>
       </c>
       <c r="G6" t="n">
-        <v>0.9714</v>
+        <v>0.9381</v>
       </c>
       <c r="H6" t="n">
-        <v>0.0068</v>
+        <v>0.0126</v>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>{'C': 10, 'epsilon': 0.1, 'kernel': 'linear'}</t>
+          <t>{'learning_rate': 0.1, 'max_depth': 3, 'n_estimators': 200}</t>
         </is>
       </c>
     </row>
@@ -1022,22 +1022,22 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>0.9811</v>
+        <v>0.9127999999999999</v>
       </c>
       <c r="D7" t="n">
-        <v>0.3203</v>
+        <v>0.0221</v>
       </c>
       <c r="E7" t="n">
-        <v>0.213</v>
+        <v>0.0158</v>
       </c>
       <c r="F7" t="n">
-        <v>0.1026</v>
+        <v>0.0005</v>
       </c>
       <c r="G7" t="n">
-        <v>0.9737</v>
+        <v>0.894</v>
       </c>
       <c r="H7" t="n">
-        <v>0.0062</v>
+        <v>0.0156</v>
       </c>
       <c r="I7" t="inlineStr">
         <is>
@@ -1055,26 +1055,26 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>0.9534</v>
+        <v>0.8925</v>
       </c>
       <c r="D8" t="n">
-        <v>0.5028</v>
+        <v>0.0246</v>
       </c>
       <c r="E8" t="n">
-        <v>0.2703</v>
+        <v>0.0177</v>
       </c>
       <c r="F8" t="n">
-        <v>0.2528</v>
+        <v>0.0005999999999999999</v>
       </c>
       <c r="G8" t="n">
-        <v>0.9550999999999999</v>
+        <v>0.8597</v>
       </c>
       <c r="H8" t="n">
-        <v>0.0152</v>
+        <v>0.0201</v>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>{'max_depth': 10, 'min_samples_split': 2, 'n_estimators': 200}</t>
+          <t>{'max_depth': None, 'min_samples_split': 2, 'n_estimators': 200}</t>
         </is>
       </c>
     </row>
@@ -1084,30 +1084,30 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Decision Tree</t>
+          <t>KNN Regression</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>0.9244</v>
+        <v>0.8647</v>
       </c>
       <c r="D9" t="n">
-        <v>0.6404</v>
+        <v>0.0275</v>
       </c>
       <c r="E9" t="n">
-        <v>0.4152</v>
+        <v>0.021</v>
       </c>
       <c r="F9" t="n">
-        <v>0.4101</v>
+        <v>0.0008</v>
       </c>
       <c r="G9" t="n">
-        <v>0.9421</v>
+        <v>0.8202</v>
       </c>
       <c r="H9" t="n">
-        <v>0.0158</v>
+        <v>0.0182</v>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>{'max_depth': 10, 'min_samples_leaf': 1, 'min_samples_split': 10}</t>
+          <t>{'metric': 'euclidean', 'n_neighbors': 3, 'weights': 'distance'}</t>
         </is>
       </c>
     </row>
@@ -1121,22 +1121,22 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>0.91</v>
+        <v>0.8248</v>
       </c>
       <c r="D10" t="n">
-        <v>0.6991000000000001</v>
+        <v>0.0313</v>
       </c>
       <c r="E10" t="n">
-        <v>0.4873</v>
+        <v>0.0237</v>
       </c>
       <c r="F10" t="n">
-        <v>0.4887</v>
+        <v>0.001</v>
       </c>
       <c r="G10" t="n">
-        <v>0.9195</v>
+        <v>0.8025</v>
       </c>
       <c r="H10" t="n">
-        <v>0.0138</v>
+        <v>0.0204</v>
       </c>
       <c r="I10" t="inlineStr">
         <is>
@@ -1150,30 +1150,30 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>KNN Regression</t>
+          <t>Decision Tree</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>0.8596</v>
+        <v>0.787</v>
       </c>
       <c r="D11" t="n">
-        <v>0.873</v>
+        <v>0.0346</v>
       </c>
       <c r="E11" t="n">
-        <v>0.5697</v>
+        <v>0.0278</v>
       </c>
       <c r="F11" t="n">
-        <v>0.7621</v>
+        <v>0.0012</v>
       </c>
       <c r="G11" t="n">
-        <v>0.8314</v>
+        <v>0.6851</v>
       </c>
       <c r="H11" t="n">
-        <v>0.0233</v>
+        <v>0.0555</v>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>{'metric': 'euclidean', 'n_neighbors': 5, 'weights': 'distance'}</t>
+          <t>{'max_depth': None, 'min_samples_leaf': 2, 'min_samples_split': 2}</t>
         </is>
       </c>
     </row>
@@ -1239,30 +1239,30 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>SVR</t>
+          <t>ElasticNet</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>0.9874000000000001</v>
+        <v>1</v>
       </c>
       <c r="D2" t="n">
-        <v>0.07099999999999999</v>
+        <v>0.0005</v>
       </c>
       <c r="E2" t="n">
-        <v>0.0419</v>
+        <v>0.0004</v>
       </c>
       <c r="F2" t="n">
-        <v>0.005</v>
+        <v>0</v>
       </c>
       <c r="G2" t="n">
-        <v>0.9792</v>
+        <v>1</v>
       </c>
       <c r="H2" t="n">
-        <v>0.0109</v>
+        <v>0</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>{'C': 10, 'epsilon': 0.01, 'kernel': 'rbf'}</t>
+          <t>{'alpha': 0.001, 'l1_ratio': 0.2}</t>
         </is>
       </c>
     </row>
@@ -1272,30 +1272,30 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Gradient Boosting</t>
+          <t>Ridge Regression</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>0.9233</v>
+        <v>1</v>
       </c>
       <c r="D3" t="n">
-        <v>0.1752</v>
+        <v>0</v>
       </c>
       <c r="E3" t="n">
-        <v>0.1228</v>
+        <v>0</v>
       </c>
       <c r="F3" t="n">
-        <v>0.0307</v>
+        <v>0</v>
       </c>
       <c r="G3" t="n">
-        <v>0.9115</v>
+        <v>1</v>
       </c>
       <c r="H3" t="n">
-        <v>0.0115</v>
+        <v>0</v>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>{'learning_rate': 0.1, 'max_depth': 3, 'n_estimators': 200}</t>
+          <t>{'alpha': 0.01}</t>
         </is>
       </c>
     </row>
@@ -1305,30 +1305,30 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Extra Trees</t>
+          <t>Lasso Regression</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>0.8829</v>
+        <v>0.999</v>
       </c>
       <c r="D4" t="n">
-        <v>0.2165</v>
+        <v>0.0024</v>
       </c>
       <c r="E4" t="n">
-        <v>0.1536</v>
+        <v>0.0018</v>
       </c>
       <c r="F4" t="n">
-        <v>0.0469</v>
+        <v>0</v>
       </c>
       <c r="G4" t="n">
-        <v>0.8642</v>
+        <v>0.9991</v>
       </c>
       <c r="H4" t="n">
-        <v>0.0165</v>
+        <v>0.0002</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>{'max_depth': None, 'min_samples_split': 2, 'n_estimators': 200}</t>
+          <t>{'alpha': 0.001}</t>
         </is>
       </c>
     </row>
@@ -1338,30 +1338,30 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Random Forest</t>
+          <t>SVR</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>0.8493000000000001</v>
+        <v>0.9976</v>
       </c>
       <c r="D5" t="n">
-        <v>0.2456</v>
+        <v>0.0037</v>
       </c>
       <c r="E5" t="n">
-        <v>0.1808</v>
+        <v>0.0029</v>
       </c>
       <c r="F5" t="n">
-        <v>0.0603</v>
+        <v>0</v>
       </c>
       <c r="G5" t="n">
-        <v>0.8087</v>
+        <v>0.9971</v>
       </c>
       <c r="H5" t="n">
-        <v>0.0152</v>
+        <v>0.0005</v>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>{'max_depth': None, 'min_samples_split': 2, 'n_estimators': 200}</t>
+          <t>{'C': 0.1, 'epsilon': 0.01, 'kernel': 'linear'}</t>
         </is>
       </c>
     </row>
@@ -1371,30 +1371,30 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Ridge Regression</t>
+          <t>Gradient Boosting</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>0.8124</v>
+        <v>0.9562</v>
       </c>
       <c r="D6" t="n">
-        <v>0.2741</v>
+        <v>0.0159</v>
       </c>
       <c r="E6" t="n">
-        <v>0.1806</v>
+        <v>0.0114</v>
       </c>
       <c r="F6" t="n">
-        <v>0.0751</v>
+        <v>0.0003</v>
       </c>
       <c r="G6" t="n">
-        <v>0.8204</v>
+        <v>0.9513</v>
       </c>
       <c r="H6" t="n">
-        <v>0.0352</v>
+        <v>0.0138</v>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>{'alpha': 0.01}</t>
+          <t>{'learning_rate': 0.1, 'max_depth': 3, 'n_estimators': 200}</t>
         </is>
       </c>
     </row>
@@ -1404,30 +1404,30 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>ElasticNet</t>
+          <t>Extra Trees</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>0.8117</v>
+        <v>0.9328</v>
       </c>
       <c r="D7" t="n">
-        <v>0.2746</v>
+        <v>0.0196</v>
       </c>
       <c r="E7" t="n">
-        <v>0.1808</v>
+        <v>0.0139</v>
       </c>
       <c r="F7" t="n">
-        <v>0.07539999999999999</v>
+        <v>0.0004</v>
       </c>
       <c r="G7" t="n">
-        <v>0.8202</v>
+        <v>0.9233</v>
       </c>
       <c r="H7" t="n">
-        <v>0.0352</v>
+        <v>0.0282</v>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>{'alpha': 0.001, 'l1_ratio': 0.8}</t>
+          <t>{'max_depth': None, 'min_samples_split': 2, 'n_estimators': 100}</t>
         </is>
       </c>
     </row>
@@ -1437,30 +1437,30 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Lasso Regression</t>
+          <t>Random Forest</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>0.8116</v>
+        <v>0.8957000000000001</v>
       </c>
       <c r="D8" t="n">
-        <v>0.2746</v>
+        <v>0.0245</v>
       </c>
       <c r="E8" t="n">
-        <v>0.1808</v>
+        <v>0.0172</v>
       </c>
       <c r="F8" t="n">
-        <v>0.07539999999999999</v>
+        <v>0.0005999999999999999</v>
       </c>
       <c r="G8" t="n">
-        <v>0.8202</v>
+        <v>0.8961</v>
       </c>
       <c r="H8" t="n">
-        <v>0.0352</v>
+        <v>0.0305</v>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>{'alpha': 0.001}</t>
+          <t>{'max_depth': None, 'min_samples_split': 2, 'n_estimators': 100}</t>
         </is>
       </c>
     </row>
@@ -1474,22 +1474,22 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>0.7189</v>
+        <v>0.8604000000000001</v>
       </c>
       <c r="D9" t="n">
-        <v>0.3355</v>
+        <v>0.0283</v>
       </c>
       <c r="E9" t="n">
-        <v>0.2629</v>
+        <v>0.0213</v>
       </c>
       <c r="F9" t="n">
-        <v>0.1125</v>
+        <v>0.0008</v>
       </c>
       <c r="G9" t="n">
-        <v>0.694</v>
+        <v>0.8336</v>
       </c>
       <c r="H9" t="n">
-        <v>0.0169</v>
+        <v>0.033</v>
       </c>
       <c r="I9" t="inlineStr">
         <is>
@@ -1507,26 +1507,26 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>0.6906</v>
+        <v>0.8438</v>
       </c>
       <c r="D10" t="n">
-        <v>0.3519</v>
+        <v>0.03</v>
       </c>
       <c r="E10" t="n">
-        <v>0.2632</v>
+        <v>0.0228</v>
       </c>
       <c r="F10" t="n">
-        <v>0.1239</v>
+        <v>0.0009</v>
       </c>
       <c r="G10" t="n">
-        <v>0.6403</v>
+        <v>0.8179999999999999</v>
       </c>
       <c r="H10" t="n">
-        <v>0.034</v>
+        <v>0.0127</v>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>{'metric': 'euclidean', 'n_neighbors': 5, 'weights': 'distance'}</t>
+          <t>{'metric': 'euclidean', 'n_neighbors': 3, 'weights': 'distance'}</t>
         </is>
       </c>
     </row>
@@ -1540,26 +1540,26 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>0.6774</v>
+        <v>0.7479</v>
       </c>
       <c r="D11" t="n">
-        <v>0.3594</v>
+        <v>0.038</v>
       </c>
       <c r="E11" t="n">
-        <v>0.2748</v>
+        <v>0.0302</v>
       </c>
       <c r="F11" t="n">
-        <v>0.1292</v>
+        <v>0.0014</v>
       </c>
       <c r="G11" t="n">
-        <v>0.5062</v>
+        <v>0.7753</v>
       </c>
       <c r="H11" t="n">
-        <v>0.0954</v>
+        <v>0.0374</v>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>{'max_depth': None, 'min_samples_leaf': 4, 'min_samples_split': 10}</t>
+          <t>{'max_depth': 10, 'min_samples_leaf': 2, 'min_samples_split': 5}</t>
         </is>
       </c>
     </row>
@@ -1625,17 +1625,17 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Ridge Regression</t>
+          <t>ElasticNet</t>
         </is>
       </c>
       <c r="C2" t="n">
         <v>1</v>
       </c>
       <c r="D2" t="n">
-        <v>0</v>
+        <v>0.0004</v>
       </c>
       <c r="E2" t="n">
-        <v>0</v>
+        <v>0.0003</v>
       </c>
       <c r="F2" t="n">
         <v>0</v>
@@ -1648,7 +1648,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>{'alpha': 0.01}</t>
+          <t>{'alpha': 0.001, 'l1_ratio': 0.2}</t>
         </is>
       </c>
     </row>
@@ -1658,17 +1658,17 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Lasso Regression</t>
+          <t>Ridge Regression</t>
         </is>
       </c>
       <c r="C3" t="n">
         <v>1</v>
       </c>
       <c r="D3" t="n">
-        <v>0.0009</v>
+        <v>0</v>
       </c>
       <c r="E3" t="n">
-        <v>0.0007</v>
+        <v>0</v>
       </c>
       <c r="F3" t="n">
         <v>0</v>
@@ -1681,7 +1681,7 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>{'alpha': 0.001}</t>
+          <t>{'alpha': 0.01}</t>
         </is>
       </c>
     </row>
@@ -1691,30 +1691,30 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>ElasticNet</t>
+          <t>Lasso Regression</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>1</v>
+        <v>0.9998</v>
       </c>
       <c r="D4" t="n">
-        <v>0.0002</v>
+        <v>0.0018</v>
       </c>
       <c r="E4" t="n">
-        <v>0.0002</v>
+        <v>0.0013</v>
       </c>
       <c r="F4" t="n">
         <v>0</v>
       </c>
       <c r="G4" t="n">
-        <v>1</v>
+        <v>0.9999</v>
       </c>
       <c r="H4" t="n">
-        <v>0</v>
+        <v>0.0001</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>{'alpha': 0.001, 'l1_ratio': 0.2}</t>
+          <t>{'alpha': 0.001}</t>
         </is>
       </c>
     </row>
@@ -1728,22 +1728,22 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>0.9991</v>
+        <v>0.9989</v>
       </c>
       <c r="D5" t="n">
-        <v>0.0045</v>
+        <v>0.0046</v>
       </c>
       <c r="E5" t="n">
-        <v>0.0034</v>
+        <v>0.0041</v>
       </c>
       <c r="F5" t="n">
         <v>0</v>
       </c>
       <c r="G5" t="n">
-        <v>0.999</v>
+        <v>0.9983</v>
       </c>
       <c r="H5" t="n">
-        <v>0.0002</v>
+        <v>0.0014</v>
       </c>
       <c r="I5" t="inlineStr">
         <is>
@@ -1761,26 +1761,26 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>0.9912</v>
+        <v>0.9611</v>
       </c>
       <c r="D6" t="n">
-        <v>0.0142</v>
+        <v>0.0281</v>
       </c>
       <c r="E6" t="n">
-        <v>0.0111</v>
+        <v>0.02</v>
       </c>
       <c r="F6" t="n">
-        <v>0.0002</v>
+        <v>0.0008</v>
       </c>
       <c r="G6" t="n">
-        <v>0.9806</v>
+        <v>0.9500999999999999</v>
       </c>
       <c r="H6" t="n">
-        <v>0.008699999999999999</v>
+        <v>0.031</v>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>{'max_depth': None, 'min_samples_split': 2, 'n_estimators': 200}</t>
+          <t>{'max_depth': 10, 'min_samples_split': 2, 'n_estimators': 100}</t>
         </is>
       </c>
     </row>
@@ -1790,30 +1790,30 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Gradient Boosting</t>
+          <t>Random Forest</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>0.9818</v>
+        <v>0.9345</v>
       </c>
       <c r="D7" t="n">
-        <v>0.0204</v>
+        <v>0.0364</v>
       </c>
       <c r="E7" t="n">
-        <v>0.0148</v>
+        <v>0.0261</v>
       </c>
       <c r="F7" t="n">
-        <v>0.0004</v>
+        <v>0.0013</v>
       </c>
       <c r="G7" t="n">
-        <v>0.9792999999999999</v>
+        <v>0.9242</v>
       </c>
       <c r="H7" t="n">
-        <v>0.0078</v>
+        <v>0.0368</v>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>{'learning_rate': 0.05, 'max_depth': 3, 'n_estimators': 200}</t>
+          <t>{'max_depth': 10, 'min_samples_split': 2, 'n_estimators': 200}</t>
         </is>
       </c>
     </row>
@@ -1823,30 +1823,30 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Random Forest</t>
+          <t>Gradient Boosting</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>0.9719</v>
+        <v>0.9257</v>
       </c>
       <c r="D8" t="n">
-        <v>0.0254</v>
+        <v>0.0388</v>
       </c>
       <c r="E8" t="n">
-        <v>0.0203</v>
+        <v>0.0297</v>
       </c>
       <c r="F8" t="n">
-        <v>0.0005999999999999999</v>
+        <v>0.0015</v>
       </c>
       <c r="G8" t="n">
-        <v>0.958</v>
+        <v>0.9357</v>
       </c>
       <c r="H8" t="n">
-        <v>0.0177</v>
+        <v>0.0494</v>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>{'max_depth': 10, 'min_samples_split': 2, 'n_estimators': 50}</t>
+          <t>{'learning_rate': 0.1, 'max_depth': 3, 'n_estimators': 200}</t>
         </is>
       </c>
     </row>
@@ -1856,30 +1856,30 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>AdaBoost</t>
+          <t>KNN Regression</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>0.9629</v>
+        <v>0.9111</v>
       </c>
       <c r="D9" t="n">
-        <v>0.0292</v>
+        <v>0.0425</v>
       </c>
       <c r="E9" t="n">
-        <v>0.0162</v>
+        <v>0.0363</v>
       </c>
       <c r="F9" t="n">
-        <v>0.0009</v>
+        <v>0.0018</v>
       </c>
       <c r="G9" t="n">
-        <v>0.9453</v>
+        <v>0.8725000000000001</v>
       </c>
       <c r="H9" t="n">
-        <v>0.0165</v>
+        <v>0.0516</v>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>{'learning_rate': 1.0, 'n_estimators': 200}</t>
+          <t>{'metric': 'manhattan', 'n_neighbors': 5, 'weights': 'distance'}</t>
         </is>
       </c>
     </row>
@@ -1889,30 +1889,30 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>KNN Regression</t>
+          <t>AdaBoost</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>0.9253</v>
+        <v>0.9023</v>
       </c>
       <c r="D10" t="n">
-        <v>0.0414</v>
+        <v>0.0445</v>
       </c>
       <c r="E10" t="n">
-        <v>0.0349</v>
+        <v>0.0338</v>
       </c>
       <c r="F10" t="n">
-        <v>0.0017</v>
+        <v>0.002</v>
       </c>
       <c r="G10" t="n">
-        <v>0.9076</v>
+        <v>0.8794</v>
       </c>
       <c r="H10" t="n">
-        <v>0.0229</v>
+        <v>0.07049999999999999</v>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>{'metric': 'manhattan', 'n_neighbors': 5, 'weights': 'distance'}</t>
+          <t>{'learning_rate': 1.0, 'n_estimators': 50}</t>
         </is>
       </c>
     </row>
@@ -1926,22 +1926,22 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>0.9162</v>
+        <v>0.8326</v>
       </c>
       <c r="D11" t="n">
-        <v>0.0439</v>
+        <v>0.0583</v>
       </c>
       <c r="E11" t="n">
-        <v>0.034</v>
+        <v>0.0475</v>
       </c>
       <c r="F11" t="n">
-        <v>0.0019</v>
+        <v>0.0034</v>
       </c>
       <c r="G11" t="n">
-        <v>0.9331</v>
+        <v>0.7931</v>
       </c>
       <c r="H11" t="n">
-        <v>0.0225</v>
+        <v>0.07099999999999999</v>
       </c>
       <c r="I11" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Adaugare pptx, finalizare documentatie si proiect
</commit_message>
<xml_diff>
--- a/rezultate_brute_modele.xlsx
+++ b/rezultate_brute_modele.xlsx
@@ -7,10 +7,10 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Atacanți_FW" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Mijlocași_MF" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Fundași_DF" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Portari_GK" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Atacanti_FW_-_Gls_90" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Mijlocasi_MF_-_GplusA" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Fundasi_DF_-_plus_-90" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Portari_GK_-_Save%" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I11"/>
+  <dimension ref="A1:G11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -427,35 +427,25 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>R²</t>
+          <t>CV R² (mean)</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>RMSE</t>
+          <t>CV R² (std)</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>MAE</t>
+          <t>CV RMSE</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>MSE</t>
+          <t>CV MAE</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
-        <is>
-          <t>CV R² (mean)</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>CV R² (std)</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
         <is>
           <t>Best Params</t>
         </is>
@@ -467,30 +457,24 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>ElasticNet</t>
+          <t>Extra Trees</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>0.9963</v>
+        <v>0.9594</v>
       </c>
       <c r="D2" t="n">
-        <v>0.0065</v>
+        <v>0.0172</v>
       </c>
       <c r="E2" t="n">
-        <v>0.0052</v>
+        <v>0.0342</v>
       </c>
       <c r="F2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G2" t="n">
-        <v>0.9913</v>
-      </c>
-      <c r="H2" t="n">
-        <v>0.0038</v>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>{'alpha': 0.001, 'l1_ratio': 0.2}</t>
+        <v>0.0214</v>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>{'max_depth': 10, 'min_samples_split': 2, 'n_estimators': 200}</t>
         </is>
       </c>
     </row>
@@ -500,30 +484,24 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Ridge Regression</t>
+          <t>Gradient Boosting</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>0.9962</v>
+        <v>0.9447</v>
       </c>
       <c r="D3" t="n">
-        <v>0.0065</v>
+        <v>0.0211</v>
       </c>
       <c r="E3" t="n">
-        <v>0.0052</v>
+        <v>0.0396</v>
       </c>
       <c r="F3" t="n">
-        <v>0</v>
-      </c>
-      <c r="G3" t="n">
-        <v>0.9913999999999999</v>
-      </c>
-      <c r="H3" t="n">
-        <v>0.0039</v>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>{'alpha': 1}</t>
+        <v>0.0264</v>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>{'learning_rate': 0.05, 'max_depth': 3, 'n_estimators': 200}</t>
         </is>
       </c>
     </row>
@@ -533,30 +511,24 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Lasso Regression</t>
+          <t>SVR</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>0.9954</v>
+        <v>0.9331</v>
       </c>
       <c r="D4" t="n">
-        <v>0.0072</v>
+        <v>0.0162</v>
       </c>
       <c r="E4" t="n">
-        <v>0.0058</v>
+        <v>0.0449</v>
       </c>
       <c r="F4" t="n">
-        <v>0.0001</v>
-      </c>
-      <c r="G4" t="n">
-        <v>0.9909</v>
-      </c>
-      <c r="H4" t="n">
-        <v>0.004</v>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>{'alpha': 0.001}</t>
+        <v>0.0279</v>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>{'C': 1, 'epsilon': 0.01, 'kernel': 'rbf'}</t>
         </is>
       </c>
     </row>
@@ -566,30 +538,24 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>SVR</t>
+          <t>Random Forest</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>0.9953</v>
+        <v>0.9320000000000001</v>
       </c>
       <c r="D5" t="n">
-        <v>0.0073</v>
+        <v>0.0205</v>
       </c>
       <c r="E5" t="n">
-        <v>0.0056</v>
+        <v>0.0444</v>
       </c>
       <c r="F5" t="n">
-        <v>0.0001</v>
-      </c>
-      <c r="G5" t="n">
-        <v>0.9903999999999999</v>
-      </c>
-      <c r="H5" t="n">
-        <v>0.0038</v>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>{'C': 0.1, 'epsilon': 0.01, 'kernel': 'linear'}</t>
+        <v>0.0301</v>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>{'max_depth': None, 'min_samples_split': 2, 'n_estimators': 50}</t>
         </is>
       </c>
     </row>
@@ -599,30 +565,24 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Gradient Boosting</t>
+          <t>Ridge Regression</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>0.9568</v>
+        <v>0.907</v>
       </c>
       <c r="D6" t="n">
-        <v>0.0221</v>
+        <v>0.06</v>
       </c>
       <c r="E6" t="n">
-        <v>0.0168</v>
+        <v>0.05</v>
       </c>
       <c r="F6" t="n">
-        <v>0.0005</v>
-      </c>
-      <c r="G6" t="n">
-        <v>0.9503</v>
-      </c>
-      <c r="H6" t="n">
-        <v>0.0105</v>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>{'learning_rate': 0.05, 'max_depth': 3, 'n_estimators': 200}</t>
+        <v>0.0345</v>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>{'alpha': 10}</t>
         </is>
       </c>
     </row>
@@ -632,30 +592,24 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Extra Trees</t>
+          <t>ElasticNet</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>0.9453</v>
+        <v>0.9062</v>
       </c>
       <c r="D7" t="n">
-        <v>0.0249</v>
+        <v>0.0616</v>
       </c>
       <c r="E7" t="n">
-        <v>0.0194</v>
+        <v>0.0502</v>
       </c>
       <c r="F7" t="n">
-        <v>0.0005999999999999999</v>
-      </c>
-      <c r="G7" t="n">
-        <v>0.9634</v>
-      </c>
-      <c r="H7" t="n">
-        <v>0.0198</v>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>{'max_depth': 10, 'min_samples_split': 2, 'n_estimators': 100}</t>
+        <v>0.0334</v>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>{'alpha': 0.01, 'l1_ratio': 0.2}</t>
         </is>
       </c>
     </row>
@@ -665,30 +619,24 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Random Forest</t>
+          <t>Lasso Regression</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>0.9316</v>
+        <v>0.904</v>
       </c>
       <c r="D8" t="n">
-        <v>0.0278</v>
+        <v>0.064</v>
       </c>
       <c r="E8" t="n">
-        <v>0.0201</v>
+        <v>0.0507</v>
       </c>
       <c r="F8" t="n">
-        <v>0.0008</v>
-      </c>
-      <c r="G8" t="n">
-        <v>0.9261</v>
-      </c>
-      <c r="H8" t="n">
-        <v>0.0201</v>
-      </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>{'max_depth': 10, 'min_samples_split': 2, 'n_estimators': 200}</t>
+        <v>0.0335</v>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>{'alpha': 0.001}</t>
         </is>
       </c>
     </row>
@@ -702,24 +650,18 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>0.9182</v>
+        <v>0.8814</v>
       </c>
       <c r="D9" t="n">
-        <v>0.0305</v>
+        <v>0.0214</v>
       </c>
       <c r="E9" t="n">
-        <v>0.0234</v>
+        <v>0.0594</v>
       </c>
       <c r="F9" t="n">
-        <v>0.0009</v>
-      </c>
-      <c r="G9" t="n">
-        <v>0.9163</v>
-      </c>
-      <c r="H9" t="n">
-        <v>0.0184</v>
-      </c>
-      <c r="I9" t="inlineStr">
+        <v>0.0434</v>
+      </c>
+      <c r="G9" t="inlineStr">
         <is>
           <t>{'learning_rate': 1.0, 'n_estimators': 200}</t>
         </is>
@@ -731,30 +673,24 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Decision Tree</t>
+          <t>KNN Regression</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>0.8459</v>
+        <v>0.8809</v>
       </c>
       <c r="D10" t="n">
-        <v>0.0418</v>
+        <v>0.0169</v>
       </c>
       <c r="E10" t="n">
-        <v>0.0339</v>
+        <v>0.0597</v>
       </c>
       <c r="F10" t="n">
-        <v>0.0017</v>
-      </c>
-      <c r="G10" t="n">
-        <v>0.8544</v>
-      </c>
-      <c r="H10" t="n">
-        <v>0.0397</v>
-      </c>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>{'max_depth': None, 'min_samples_leaf': 1, 'min_samples_split': 2}</t>
+        <v>0.0461</v>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>{'metric': 'manhattan', 'n_neighbors': 5, 'weights': 'distance'}</t>
         </is>
       </c>
     </row>
@@ -764,30 +700,24 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>KNN Regression</t>
+          <t>Decision Tree</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>0.7766999999999999</v>
+        <v>0.8651</v>
       </c>
       <c r="D11" t="n">
-        <v>0.0503</v>
+        <v>0.0251</v>
       </c>
       <c r="E11" t="n">
-        <v>0.0372</v>
+        <v>0.06320000000000001</v>
       </c>
       <c r="F11" t="n">
-        <v>0.0025</v>
-      </c>
-      <c r="G11" t="n">
-        <v>0.8114</v>
-      </c>
-      <c r="H11" t="n">
-        <v>0.0311</v>
-      </c>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>{'metric': 'euclidean', 'n_neighbors': 5, 'weights': 'distance'}</t>
+        <v>0.0455</v>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>{'max_depth': 10, 'min_samples_leaf': 2, 'min_samples_split': 10}</t>
         </is>
       </c>
     </row>
@@ -802,7 +732,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I11"/>
+  <dimension ref="A1:G11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -813,35 +743,25 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>R²</t>
+          <t>CV R² (mean)</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>RMSE</t>
+          <t>CV R² (std)</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>MAE</t>
+          <t>CV RMSE</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>MSE</t>
+          <t>CV MAE</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
-        <is>
-          <t>CV R² (mean)</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>CV R² (std)</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
         <is>
           <t>Best Params</t>
         </is>
@@ -857,26 +777,20 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>1</v>
+        <v>0.7454</v>
       </c>
       <c r="D2" t="n">
-        <v>0</v>
+        <v>0.0366</v>
       </c>
       <c r="E2" t="n">
-        <v>0</v>
+        <v>2.0343</v>
       </c>
       <c r="F2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G2" t="n">
-        <v>1</v>
-      </c>
-      <c r="H2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>{'alpha': 0.01}</t>
+        <v>1.4977</v>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>{'alpha': 10}</t>
         </is>
       </c>
     </row>
@@ -890,26 +804,20 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>0.9999</v>
+        <v>0.7452</v>
       </c>
       <c r="D3" t="n">
-        <v>0.0005999999999999999</v>
+        <v>0.0371</v>
       </c>
       <c r="E3" t="n">
-        <v>0.0005</v>
+        <v>2.0348</v>
       </c>
       <c r="F3" t="n">
-        <v>0</v>
-      </c>
-      <c r="G3" t="n">
-        <v>0.9999</v>
-      </c>
-      <c r="H3" t="n">
-        <v>0</v>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>{'alpha': 0.001, 'l1_ratio': 0.2}</t>
+        <v>1.5005</v>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>{'alpha': 0.01, 'l1_ratio': 0.2}</t>
         </is>
       </c>
     </row>
@@ -923,24 +831,18 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>0.9986</v>
+        <v>0.745</v>
       </c>
       <c r="D4" t="n">
-        <v>0.0028</v>
+        <v>0.0375</v>
       </c>
       <c r="E4" t="n">
-        <v>0.0023</v>
+        <v>2.0355</v>
       </c>
       <c r="F4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G4" t="n">
-        <v>0.9986</v>
-      </c>
-      <c r="H4" t="n">
-        <v>0.0002</v>
-      </c>
-      <c r="I4" t="inlineStr">
+        <v>1.5036</v>
+      </c>
+      <c r="G4" t="inlineStr">
         <is>
           <t>{'alpha': 0.001}</t>
         </is>
@@ -952,30 +854,24 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>SVR</t>
+          <t>Gradient Boosting</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>0.9963</v>
+        <v>0.7398</v>
       </c>
       <c r="D5" t="n">
-        <v>0.0045</v>
+        <v>0.0531</v>
       </c>
       <c r="E5" t="n">
-        <v>0.0036</v>
+        <v>2.0541</v>
       </c>
       <c r="F5" t="n">
-        <v>0</v>
-      </c>
-      <c r="G5" t="n">
-        <v>0.9961</v>
-      </c>
-      <c r="H5" t="n">
-        <v>0.0007</v>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>{'C': 0.1, 'epsilon': 0.01, 'kernel': 'linear'}</t>
+        <v>1.3551</v>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>{'learning_rate': 0.05, 'max_depth': 3, 'n_estimators': 200}</t>
         </is>
       </c>
     </row>
@@ -985,30 +881,24 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Gradient Boosting</t>
+          <t>SVR</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>0.9664</v>
+        <v>0.7314000000000001</v>
       </c>
       <c r="D6" t="n">
-        <v>0.0137</v>
+        <v>0.0351</v>
       </c>
       <c r="E6" t="n">
-        <v>0.009900000000000001</v>
+        <v>2.0915</v>
       </c>
       <c r="F6" t="n">
-        <v>0.0002</v>
-      </c>
-      <c r="G6" t="n">
-        <v>0.9381</v>
-      </c>
-      <c r="H6" t="n">
-        <v>0.0126</v>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>{'learning_rate': 0.1, 'max_depth': 3, 'n_estimators': 200}</t>
+        <v>1.4641</v>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>{'C': 10, 'epsilon': 0.5, 'kernel': 'linear'}</t>
         </is>
       </c>
     </row>
@@ -1018,30 +908,24 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Extra Trees</t>
+          <t>Random Forest</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>0.9127999999999999</v>
+        <v>0.7282</v>
       </c>
       <c r="D7" t="n">
-        <v>0.0221</v>
+        <v>0.07340000000000001</v>
       </c>
       <c r="E7" t="n">
-        <v>0.0158</v>
+        <v>2.0931</v>
       </c>
       <c r="F7" t="n">
-        <v>0.0005</v>
-      </c>
-      <c r="G7" t="n">
-        <v>0.894</v>
-      </c>
-      <c r="H7" t="n">
-        <v>0.0156</v>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>{'max_depth': None, 'min_samples_split': 2, 'n_estimators': 200}</t>
+        <v>1.3601</v>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>{'max_depth': 10, 'min_samples_split': 2, 'n_estimators': 50}</t>
         </is>
       </c>
     </row>
@@ -1051,30 +935,24 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Random Forest</t>
+          <t>Extra Trees</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>0.8925</v>
+        <v>0.7169</v>
       </c>
       <c r="D8" t="n">
-        <v>0.0246</v>
+        <v>0.0463</v>
       </c>
       <c r="E8" t="n">
-        <v>0.0177</v>
+        <v>2.1459</v>
       </c>
       <c r="F8" t="n">
-        <v>0.0005999999999999999</v>
-      </c>
-      <c r="G8" t="n">
-        <v>0.8597</v>
-      </c>
-      <c r="H8" t="n">
-        <v>0.0201</v>
-      </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>{'max_depth': None, 'min_samples_split': 2, 'n_estimators': 200}</t>
+        <v>1.4094</v>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>{'max_depth': None, 'min_samples_split': 5, 'n_estimators': 50}</t>
         </is>
       </c>
     </row>
@@ -1088,26 +966,20 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>0.8647</v>
+        <v>0.6705</v>
       </c>
       <c r="D9" t="n">
-        <v>0.0275</v>
+        <v>0.0392</v>
       </c>
       <c r="E9" t="n">
-        <v>0.021</v>
+        <v>2.3208</v>
       </c>
       <c r="F9" t="n">
-        <v>0.0008</v>
-      </c>
-      <c r="G9" t="n">
-        <v>0.8202</v>
-      </c>
-      <c r="H9" t="n">
-        <v>0.0182</v>
-      </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>{'metric': 'euclidean', 'n_neighbors': 3, 'weights': 'distance'}</t>
+        <v>1.5499</v>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>{'metric': 'euclidean', 'n_neighbors': 10, 'weights': 'distance'}</t>
         </is>
       </c>
     </row>
@@ -1121,26 +993,20 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>0.8248</v>
+        <v>0.6667</v>
       </c>
       <c r="D10" t="n">
-        <v>0.0313</v>
+        <v>0.0654</v>
       </c>
       <c r="E10" t="n">
-        <v>0.0237</v>
+        <v>2.3269</v>
       </c>
       <c r="F10" t="n">
-        <v>0.001</v>
-      </c>
-      <c r="G10" t="n">
-        <v>0.8025</v>
-      </c>
-      <c r="H10" t="n">
-        <v>0.0204</v>
-      </c>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>{'learning_rate': 1.0, 'n_estimators': 200}</t>
+        <v>1.7005</v>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>{'learning_rate': 0.1, 'n_estimators': 100}</t>
         </is>
       </c>
     </row>
@@ -1154,26 +1020,20 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>0.787</v>
+        <v>0.6317</v>
       </c>
       <c r="D11" t="n">
-        <v>0.0346</v>
+        <v>0.1081</v>
       </c>
       <c r="E11" t="n">
-        <v>0.0278</v>
+        <v>2.4201</v>
       </c>
       <c r="F11" t="n">
-        <v>0.0012</v>
-      </c>
-      <c r="G11" t="n">
-        <v>0.6851</v>
-      </c>
-      <c r="H11" t="n">
-        <v>0.0555</v>
-      </c>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>{'max_depth': None, 'min_samples_leaf': 2, 'min_samples_split': 2}</t>
+        <v>1.5739</v>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>{'max_depth': 5, 'min_samples_leaf': 4, 'min_samples_split': 10}</t>
         </is>
       </c>
     </row>
@@ -1188,7 +1048,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I11"/>
+  <dimension ref="A1:G11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1199,35 +1059,25 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>R²</t>
+          <t>CV R² (mean)</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>RMSE</t>
+          <t>CV R² (std)</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>MAE</t>
+          <t>CV RMSE</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>MSE</t>
+          <t>CV MAE</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
-        <is>
-          <t>CV R² (mean)</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>CV R² (std)</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
         <is>
           <t>Best Params</t>
         </is>
@@ -1243,26 +1093,20 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>1</v>
+        <v>0.9174</v>
       </c>
       <c r="D2" t="n">
-        <v>0.0005</v>
+        <v>0.0162</v>
       </c>
       <c r="E2" t="n">
-        <v>0.0004</v>
+        <v>0.2055</v>
       </c>
       <c r="F2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G2" t="n">
-        <v>1</v>
-      </c>
-      <c r="H2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>{'alpha': 0.001, 'l1_ratio': 0.2}</t>
+        <v>0.1621</v>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>{'alpha': 0.01, 'l1_ratio': 0.2}</t>
         </is>
       </c>
     </row>
@@ -1272,30 +1116,24 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Ridge Regression</t>
+          <t>SVR</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>1</v>
+        <v>0.9173</v>
       </c>
       <c r="D3" t="n">
-        <v>0</v>
+        <v>0.0162</v>
       </c>
       <c r="E3" t="n">
-        <v>0</v>
+        <v>0.2055</v>
       </c>
       <c r="F3" t="n">
-        <v>0</v>
-      </c>
-      <c r="G3" t="n">
-        <v>1</v>
-      </c>
-      <c r="H3" t="n">
-        <v>0</v>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>{'alpha': 0.01}</t>
+        <v>0.1623</v>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>{'C': 1, 'epsilon': 0.1, 'kernel': 'linear'}</t>
         </is>
       </c>
     </row>
@@ -1309,24 +1147,18 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>0.999</v>
+        <v>0.9172</v>
       </c>
       <c r="D4" t="n">
-        <v>0.0024</v>
+        <v>0.0157</v>
       </c>
       <c r="E4" t="n">
-        <v>0.0018</v>
+        <v>0.2057</v>
       </c>
       <c r="F4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G4" t="n">
-        <v>0.9991</v>
-      </c>
-      <c r="H4" t="n">
-        <v>0.0002</v>
-      </c>
-      <c r="I4" t="inlineStr">
+        <v>0.1625</v>
+      </c>
+      <c r="G4" t="inlineStr">
         <is>
           <t>{'alpha': 0.001}</t>
         </is>
@@ -1338,30 +1170,24 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>SVR</t>
+          <t>Ridge Regression</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>0.9976</v>
+        <v>0.9171</v>
       </c>
       <c r="D5" t="n">
-        <v>0.0037</v>
+        <v>0.0156</v>
       </c>
       <c r="E5" t="n">
-        <v>0.0029</v>
+        <v>0.2059</v>
       </c>
       <c r="F5" t="n">
-        <v>0</v>
-      </c>
-      <c r="G5" t="n">
-        <v>0.9971</v>
-      </c>
-      <c r="H5" t="n">
-        <v>0.0005</v>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>{'C': 0.1, 'epsilon': 0.01, 'kernel': 'linear'}</t>
+        <v>0.1626</v>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>{'alpha': 1}</t>
         </is>
       </c>
     </row>
@@ -1371,30 +1197,24 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Gradient Boosting</t>
+          <t>Extra Trees</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>0.9562</v>
+        <v>0.9157999999999999</v>
       </c>
       <c r="D6" t="n">
-        <v>0.0159</v>
+        <v>0.0198</v>
       </c>
       <c r="E6" t="n">
-        <v>0.0114</v>
+        <v>0.2071</v>
       </c>
       <c r="F6" t="n">
-        <v>0.0003</v>
-      </c>
-      <c r="G6" t="n">
-        <v>0.9513</v>
-      </c>
-      <c r="H6" t="n">
-        <v>0.0138</v>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>{'learning_rate': 0.1, 'max_depth': 3, 'n_estimators': 200}</t>
+        <v>0.1615</v>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>{'max_depth': 10, 'min_samples_split': 5, 'n_estimators': 200}</t>
         </is>
       </c>
     </row>
@@ -1404,30 +1224,24 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Extra Trees</t>
+          <t>Gradient Boosting</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>0.9328</v>
+        <v>0.9123</v>
       </c>
       <c r="D7" t="n">
-        <v>0.0196</v>
+        <v>0.0146</v>
       </c>
       <c r="E7" t="n">
-        <v>0.0139</v>
+        <v>0.2123</v>
       </c>
       <c r="F7" t="n">
-        <v>0.0004</v>
-      </c>
-      <c r="G7" t="n">
-        <v>0.9233</v>
-      </c>
-      <c r="H7" t="n">
-        <v>0.0282</v>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>{'max_depth': None, 'min_samples_split': 2, 'n_estimators': 100}</t>
+        <v>0.1652</v>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>{'learning_rate': 0.05, 'max_depth': 3, 'n_estimators': 100}</t>
         </is>
       </c>
     </row>
@@ -1441,26 +1255,20 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>0.8957000000000001</v>
+        <v>0.9076</v>
       </c>
       <c r="D8" t="n">
-        <v>0.0245</v>
+        <v>0.0204</v>
       </c>
       <c r="E8" t="n">
-        <v>0.0172</v>
+        <v>0.217</v>
       </c>
       <c r="F8" t="n">
-        <v>0.0005999999999999999</v>
-      </c>
-      <c r="G8" t="n">
-        <v>0.8961</v>
-      </c>
-      <c r="H8" t="n">
-        <v>0.0305</v>
-      </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>{'max_depth': None, 'min_samples_split': 2, 'n_estimators': 100}</t>
+        <v>0.1668</v>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>{'max_depth': 5, 'min_samples_split': 2, 'n_estimators': 200}</t>
         </is>
       </c>
     </row>
@@ -1474,26 +1282,20 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>0.8604000000000001</v>
+        <v>0.9016</v>
       </c>
       <c r="D9" t="n">
-        <v>0.0283</v>
+        <v>0.0229</v>
       </c>
       <c r="E9" t="n">
-        <v>0.0213</v>
+        <v>0.2239</v>
       </c>
       <c r="F9" t="n">
-        <v>0.0008</v>
-      </c>
-      <c r="G9" t="n">
-        <v>0.8336</v>
-      </c>
-      <c r="H9" t="n">
-        <v>0.033</v>
-      </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>{'learning_rate': 1.0, 'n_estimators': 200}</t>
+        <v>0.1769</v>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>{'learning_rate': 0.1, 'n_estimators': 200}</t>
         </is>
       </c>
     </row>
@@ -1503,30 +1305,24 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>KNN Regression</t>
+          <t>Decision Tree</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>0.8438</v>
+        <v>0.8718</v>
       </c>
       <c r="D10" t="n">
-        <v>0.03</v>
+        <v>0.0188</v>
       </c>
       <c r="E10" t="n">
-        <v>0.0228</v>
+        <v>0.2561</v>
       </c>
       <c r="F10" t="n">
-        <v>0.0009</v>
-      </c>
-      <c r="G10" t="n">
-        <v>0.8179999999999999</v>
-      </c>
-      <c r="H10" t="n">
-        <v>0.0127</v>
-      </c>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>{'metric': 'euclidean', 'n_neighbors': 3, 'weights': 'distance'}</t>
+        <v>0.1956</v>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>{'max_depth': 5, 'min_samples_leaf': 2, 'min_samples_split': 10}</t>
         </is>
       </c>
     </row>
@@ -1536,30 +1332,24 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Decision Tree</t>
+          <t>KNN Regression</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>0.7479</v>
+        <v>0.8073</v>
       </c>
       <c r="D11" t="n">
-        <v>0.038</v>
+        <v>0.0563</v>
       </c>
       <c r="E11" t="n">
-        <v>0.0302</v>
+        <v>0.3119</v>
       </c>
       <c r="F11" t="n">
-        <v>0.0014</v>
-      </c>
-      <c r="G11" t="n">
-        <v>0.7753</v>
-      </c>
-      <c r="H11" t="n">
-        <v>0.0374</v>
-      </c>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>{'max_depth': 10, 'min_samples_leaf': 2, 'min_samples_split': 5}</t>
+        <v>0.2383</v>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>{'metric': 'manhattan', 'n_neighbors': 7, 'weights': 'distance'}</t>
         </is>
       </c>
     </row>
@@ -1574,7 +1364,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I11"/>
+  <dimension ref="A1:G11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1585,35 +1375,25 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>R²</t>
+          <t>CV R² (mean)</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>RMSE</t>
+          <t>CV R² (std)</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>MAE</t>
+          <t>CV RMSE</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>MSE</t>
+          <t>CV MAE</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
-        <is>
-          <t>CV R² (mean)</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>CV R² (std)</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
         <is>
           <t>Best Params</t>
         </is>
@@ -1625,30 +1405,24 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>ElasticNet</t>
+          <t>SVR</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>1</v>
+        <v>0.8144</v>
       </c>
       <c r="D2" t="n">
-        <v>0.0004</v>
+        <v>0.0384</v>
       </c>
       <c r="E2" t="n">
-        <v>0.0003</v>
+        <v>1.8763</v>
       </c>
       <c r="F2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G2" t="n">
-        <v>1</v>
-      </c>
-      <c r="H2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>{'alpha': 0.001, 'l1_ratio': 0.2}</t>
+        <v>1.4586</v>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>{'C': 10, 'epsilon': 0.5, 'kernel': 'linear'}</t>
         </is>
       </c>
     </row>
@@ -1658,30 +1432,24 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Ridge Regression</t>
+          <t>Lasso Regression</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>1</v>
+        <v>0.8097</v>
       </c>
       <c r="D3" t="n">
-        <v>0</v>
+        <v>0.0324</v>
       </c>
       <c r="E3" t="n">
-        <v>0</v>
+        <v>1.91</v>
       </c>
       <c r="F3" t="n">
-        <v>0</v>
-      </c>
-      <c r="G3" t="n">
-        <v>1</v>
-      </c>
-      <c r="H3" t="n">
-        <v>0</v>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>{'alpha': 0.01}</t>
+        <v>1.4582</v>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>{'alpha': 0.1}</t>
         </is>
       </c>
     </row>
@@ -1691,30 +1459,24 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Lasso Regression</t>
+          <t>ElasticNet</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>0.9998</v>
+        <v>0.8096</v>
       </c>
       <c r="D4" t="n">
-        <v>0.0018</v>
+        <v>0.0459</v>
       </c>
       <c r="E4" t="n">
-        <v>0.0013</v>
+        <v>1.8969</v>
       </c>
       <c r="F4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G4" t="n">
-        <v>0.9999</v>
-      </c>
-      <c r="H4" t="n">
-        <v>0.0001</v>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>{'alpha': 0.001}</t>
+        <v>1.4686</v>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>{'alpha': 0.01, 'l1_ratio': 0.5}</t>
         </is>
       </c>
     </row>
@@ -1724,30 +1486,24 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>SVR</t>
+          <t>Ridge Regression</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>0.9989</v>
+        <v>0.8091</v>
       </c>
       <c r="D5" t="n">
-        <v>0.0046</v>
+        <v>0.0418</v>
       </c>
       <c r="E5" t="n">
-        <v>0.0041</v>
+        <v>1.9079</v>
       </c>
       <c r="F5" t="n">
-        <v>0</v>
-      </c>
-      <c r="G5" t="n">
-        <v>0.9983</v>
-      </c>
-      <c r="H5" t="n">
-        <v>0.0014</v>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>{'C': 0.1, 'epsilon': 0.01, 'kernel': 'linear'}</t>
+        <v>1.4698</v>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>{'alpha': 1}</t>
         </is>
       </c>
     </row>
@@ -1761,26 +1517,20 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>0.9611</v>
+        <v>0.5601</v>
       </c>
       <c r="D6" t="n">
-        <v>0.0281</v>
+        <v>0.1163</v>
       </c>
       <c r="E6" t="n">
-        <v>0.02</v>
+        <v>2.9307</v>
       </c>
       <c r="F6" t="n">
-        <v>0.0008</v>
-      </c>
-      <c r="G6" t="n">
-        <v>0.9500999999999999</v>
-      </c>
-      <c r="H6" t="n">
-        <v>0.031</v>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>{'max_depth': 10, 'min_samples_split': 2, 'n_estimators': 100}</t>
+        <v>2.3157</v>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>{'max_depth': 10, 'min_samples_split': 2, 'n_estimators': 50}</t>
         </is>
       </c>
     </row>
@@ -1790,30 +1540,24 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Random Forest</t>
+          <t>Gradient Boosting</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>0.9345</v>
+        <v>0.5538</v>
       </c>
       <c r="D7" t="n">
-        <v>0.0364</v>
+        <v>0.0886</v>
       </c>
       <c r="E7" t="n">
-        <v>0.0261</v>
+        <v>2.945</v>
       </c>
       <c r="F7" t="n">
-        <v>0.0013</v>
-      </c>
-      <c r="G7" t="n">
-        <v>0.9242</v>
-      </c>
-      <c r="H7" t="n">
-        <v>0.0368</v>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>{'max_depth': 10, 'min_samples_split': 2, 'n_estimators': 200}</t>
+        <v>2.3498</v>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>{'learning_rate': 0.1, 'max_depth': 3, 'n_estimators': 100}</t>
         </is>
       </c>
     </row>
@@ -1823,30 +1567,24 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Gradient Boosting</t>
+          <t>Random Forest</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>0.9257</v>
+        <v>0.5179</v>
       </c>
       <c r="D8" t="n">
-        <v>0.0388</v>
+        <v>0.0672</v>
       </c>
       <c r="E8" t="n">
-        <v>0.0297</v>
+        <v>3.0835</v>
       </c>
       <c r="F8" t="n">
-        <v>0.0015</v>
-      </c>
-      <c r="G8" t="n">
-        <v>0.9357</v>
-      </c>
-      <c r="H8" t="n">
-        <v>0.0494</v>
-      </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>{'learning_rate': 0.1, 'max_depth': 3, 'n_estimators': 200}</t>
+        <v>2.4735</v>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>{'max_depth': None, 'min_samples_split': 5, 'n_estimators': 50}</t>
         </is>
       </c>
     </row>
@@ -1856,30 +1594,24 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>KNN Regression</t>
+          <t>AdaBoost</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>0.9111</v>
+        <v>0.4624</v>
       </c>
       <c r="D9" t="n">
-        <v>0.0425</v>
+        <v>0.0654</v>
       </c>
       <c r="E9" t="n">
-        <v>0.0363</v>
+        <v>3.2192</v>
       </c>
       <c r="F9" t="n">
-        <v>0.0018</v>
-      </c>
-      <c r="G9" t="n">
-        <v>0.8725000000000001</v>
-      </c>
-      <c r="H9" t="n">
-        <v>0.0516</v>
-      </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>{'metric': 'manhattan', 'n_neighbors': 5, 'weights': 'distance'}</t>
+        <v>2.5449</v>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>{'learning_rate': 1.0, 'n_estimators': 200}</t>
         </is>
       </c>
     </row>
@@ -1889,30 +1621,24 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>AdaBoost</t>
+          <t>KNN Regression</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>0.9023</v>
+        <v>0.3952</v>
       </c>
       <c r="D10" t="n">
-        <v>0.0445</v>
+        <v>0.098</v>
       </c>
       <c r="E10" t="n">
-        <v>0.0338</v>
+        <v>3.4208</v>
       </c>
       <c r="F10" t="n">
-        <v>0.002</v>
-      </c>
-      <c r="G10" t="n">
-        <v>0.8794</v>
-      </c>
-      <c r="H10" t="n">
-        <v>0.07049999999999999</v>
-      </c>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>{'learning_rate': 1.0, 'n_estimators': 50}</t>
+        <v>2.7108</v>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>{'metric': 'euclidean', 'n_neighbors': 7, 'weights': 'distance'}</t>
         </is>
       </c>
     </row>
@@ -1926,26 +1652,20 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>0.8326</v>
+        <v>0.3556</v>
       </c>
       <c r="D11" t="n">
-        <v>0.0583</v>
+        <v>0.0486</v>
       </c>
       <c r="E11" t="n">
-        <v>0.0475</v>
+        <v>3.5414</v>
       </c>
       <c r="F11" t="n">
-        <v>0.0034</v>
-      </c>
-      <c r="G11" t="n">
-        <v>0.7931</v>
-      </c>
-      <c r="H11" t="n">
-        <v>0.07099999999999999</v>
-      </c>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>{'max_depth': 5, 'min_samples_leaf': 2, 'min_samples_split': 2}</t>
+        <v>2.8626</v>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>{'max_depth': 10, 'min_samples_leaf': 1, 'min_samples_split': 10}</t>
         </is>
       </c>
     </row>

</xml_diff>